<commit_message>
rename S3 S4 to S1 S2
</commit_message>
<xml_diff>
--- a/data/Omicron_BA2.xlsx
+++ b/data/Omicron_BA2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\omicron\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - kanggle\XMU\likangguo\other\github\zhuhai_omicron\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4048DD8-5A22-43C8-9E33-C1FB44BAEC9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{945E2ACE-0972-404A-B984-B38B58134F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="44">
   <si>
     <t>id</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -196,6 +196,10 @@
   </si>
   <si>
     <t>vaccinelastdate</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>datereported</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -669,7 +673,7 @@
         <v>7</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="J1" s="6" t="s">
         <v>9</v>
@@ -710,10 +714,10 @@
         <v>44631</v>
       </c>
       <c r="H2" s="10">
-        <v>44631</v>
+        <v>44631.786805555559</v>
       </c>
       <c r="I2" s="10">
-        <v>44631</v>
+        <v>44631.951388888891</v>
       </c>
       <c r="J2" s="4">
         <v>3</v>
@@ -754,10 +758,10 @@
         <v>44633</v>
       </c>
       <c r="H3" s="10">
-        <v>44633</v>
+        <v>44633.929166666669</v>
       </c>
       <c r="I3" s="10">
-        <v>44633</v>
+        <v>44634.31659722222</v>
       </c>
       <c r="J3" s="1">
         <v>3</v>
@@ -798,10 +802,10 @@
         <v>44633</v>
       </c>
       <c r="H4" s="10">
-        <v>44633</v>
+        <v>44634.131944444445</v>
       </c>
       <c r="I4" s="10">
-        <v>44633</v>
+        <v>44634.468738425923</v>
       </c>
       <c r="J4" s="1">
         <v>3</v>
@@ -842,10 +846,10 @@
         <v>44634</v>
       </c>
       <c r="H5" s="10">
-        <v>44634</v>
+        <v>44634.958333333336</v>
       </c>
       <c r="I5" s="10">
-        <v>44634</v>
+        <v>44635.300555555557</v>
       </c>
       <c r="J5" s="1">
         <v>2</v>
@@ -886,10 +890,10 @@
         <v>44635</v>
       </c>
       <c r="H6" s="10">
-        <v>44635</v>
+        <v>44635.806944444441</v>
       </c>
       <c r="I6" s="10">
-        <v>44635</v>
+        <v>44635.934907407405</v>
       </c>
       <c r="J6" s="1">
         <v>3</v>
@@ -930,10 +934,10 @@
         <v>44635</v>
       </c>
       <c r="H7" s="10">
-        <v>44635</v>
+        <v>44635.933333333334</v>
       </c>
       <c r="I7" s="10">
-        <v>44635</v>
+        <v>44636.29173611111</v>
       </c>
       <c r="J7" s="1">
         <v>2</v>
@@ -974,10 +978,10 @@
         <v>44635</v>
       </c>
       <c r="H8" s="10">
-        <v>44635</v>
+        <v>44635.772222222222</v>
       </c>
       <c r="I8" s="10">
-        <v>44635</v>
+        <v>44636.294895833336</v>
       </c>
       <c r="J8" s="1">
         <v>3</v>
@@ -1018,10 +1022,10 @@
         <v>44635</v>
       </c>
       <c r="H9" s="10">
-        <v>44635</v>
+        <v>44636.12222222222</v>
       </c>
       <c r="I9" s="10">
-        <v>44635</v>
+        <v>44636.309178240743</v>
       </c>
       <c r="J9" s="1">
         <v>2</v>
@@ -1062,10 +1066,10 @@
         <v>44635</v>
       </c>
       <c r="H10" s="10">
-        <v>44635</v>
+        <v>44636.261111111111</v>
       </c>
       <c r="I10" s="10">
-        <v>44635</v>
+        <v>44636.510717592595</v>
       </c>
       <c r="J10" s="1">
         <v>3</v>
@@ -1106,10 +1110,10 @@
         <v>44635</v>
       </c>
       <c r="H11" s="10">
-        <v>44635</v>
+        <v>44636.73333333333</v>
       </c>
       <c r="I11" s="10">
-        <v>44635</v>
+        <v>44636.883715277778</v>
       </c>
       <c r="J11" s="1">
         <v>3</v>
@@ -1150,10 +1154,10 @@
         <v>44636</v>
       </c>
       <c r="H12" s="10">
-        <v>44636</v>
+        <v>44637.155555555553</v>
       </c>
       <c r="I12" s="10">
-        <v>44636</v>
+        <v>44637.483298611114</v>
       </c>
       <c r="J12" s="1">
         <v>3</v>
@@ -1194,10 +1198,10 @@
         <v>44637</v>
       </c>
       <c r="H13" s="10">
-        <v>44637</v>
+        <v>44637.962500000001</v>
       </c>
       <c r="I13" s="10">
-        <v>44637</v>
+        <v>44638.348622685182</v>
       </c>
       <c r="J13" s="1">
         <v>2</v>
@@ -1238,10 +1242,10 @@
         <v>44638</v>
       </c>
       <c r="H14" s="10">
-        <v>44638</v>
+        <v>44638.314583333333</v>
       </c>
       <c r="I14" s="10">
-        <v>44638</v>
+        <v>44638.617407407408</v>
       </c>
       <c r="J14" s="1">
         <v>2</v>
@@ -1282,10 +1286,10 @@
         <v>44638</v>
       </c>
       <c r="H15" s="10">
-        <v>44638</v>
+        <v>44638.492361111108</v>
       </c>
       <c r="I15" s="10">
-        <v>44638</v>
+        <v>44638.740370370368</v>
       </c>
       <c r="J15" s="1">
         <v>2</v>
@@ -1326,10 +1330,10 @@
         <v>44638</v>
       </c>
       <c r="H16" s="10">
-        <v>44638</v>
+        <v>44639.061805555553</v>
       </c>
       <c r="I16" s="10">
-        <v>44638</v>
+        <v>44639.417210648149</v>
       </c>
       <c r="J16" s="1">
         <v>2</v>
@@ -1370,10 +1374,10 @@
         <v>44638</v>
       </c>
       <c r="H17" s="10">
-        <v>44638</v>
+        <v>44638.875</v>
       </c>
       <c r="I17" s="10">
-        <v>44638</v>
+        <v>44639.418321759258</v>
       </c>
       <c r="J17" s="1">
         <v>2</v>
@@ -1414,10 +1418,10 @@
         <v>44638</v>
       </c>
       <c r="H18" s="10">
-        <v>44638</v>
+        <v>44639.109027777777</v>
       </c>
       <c r="I18" s="10">
-        <v>44638</v>
+        <v>44639.419502314813</v>
       </c>
       <c r="J18" s="1">
         <v>2</v>
@@ -1458,10 +1462,10 @@
         <v>44638</v>
       </c>
       <c r="H19" s="10">
-        <v>44638</v>
+        <v>44639.54583333333</v>
       </c>
       <c r="I19" s="10">
-        <v>44638</v>
+        <v>44639.806770833333</v>
       </c>
       <c r="J19" s="1">
         <v>3</v>
@@ -1502,10 +1506,10 @@
         <v>44639</v>
       </c>
       <c r="H20" s="10">
-        <v>44639</v>
+        <v>44639.90347222222</v>
       </c>
       <c r="I20" s="10">
-        <v>44639</v>
+        <v>44640.345046296294</v>
       </c>
       <c r="J20" s="1">
         <v>2</v>
@@ -1546,10 +1550,10 @@
         <v>44638</v>
       </c>
       <c r="H21" s="10">
-        <v>44638</v>
+        <v>44640.314583333333</v>
       </c>
       <c r="I21" s="10">
-        <v>44638</v>
+        <v>44640.641643518517</v>
       </c>
       <c r="J21" s="1">
         <v>2</v>
@@ -1590,10 +1594,10 @@
         <v>44640</v>
       </c>
       <c r="H22" s="10">
-        <v>44640</v>
+        <v>44641.01667824074</v>
       </c>
       <c r="I22" s="10">
-        <v>44640</v>
+        <v>44641.357430555552</v>
       </c>
       <c r="J22" s="1">
         <v>3</v>
@@ -1634,10 +1638,10 @@
         <v>44640</v>
       </c>
       <c r="H23" s="10">
-        <v>44640</v>
+        <v>44641.015289351853</v>
       </c>
       <c r="I23" s="10">
-        <v>44640</v>
+        <v>44641.358784722222</v>
       </c>
       <c r="J23" s="1">
         <v>2</v>
@@ -1678,10 +1682,10 @@
         <v>44649</v>
       </c>
       <c r="H24" s="10">
-        <v>44649</v>
+        <v>44650.113194444442</v>
       </c>
       <c r="I24" s="10">
-        <v>44649</v>
+        <v>44650.359386574077</v>
       </c>
       <c r="J24" s="1">
         <v>3</v>
@@ -1722,10 +1726,10 @@
         <v>44649</v>
       </c>
       <c r="H25" s="10">
-        <v>44649</v>
+        <v>44650.109027777777</v>
       </c>
       <c r="I25" s="10">
-        <v>44649</v>
+        <v>44650.361064814817</v>
       </c>
       <c r="J25" s="1">
         <v>3</v>
@@ -1766,10 +1770,10 @@
         <v>44649</v>
       </c>
       <c r="H26" s="10">
-        <v>44649</v>
+        <v>44650.541666666664</v>
       </c>
       <c r="I26" s="10">
-        <v>44649</v>
+        <v>44650.695011574076</v>
       </c>
       <c r="J26" s="1">
         <v>2</v>
@@ -1810,10 +1814,10 @@
         <v>44649</v>
       </c>
       <c r="H27" s="10">
-        <v>44649</v>
+        <v>44650.284722222219</v>
       </c>
       <c r="I27" s="10">
-        <v>44649</v>
+        <v>44650.697939814818</v>
       </c>
       <c r="J27" s="1">
         <v>2</v>
@@ -1854,10 +1858,10 @@
         <v>44650</v>
       </c>
       <c r="H28" s="10">
-        <v>44650</v>
+        <v>44650.6875</v>
       </c>
       <c r="I28" s="10">
-        <v>44650</v>
+        <v>44650.892291666663</v>
       </c>
       <c r="J28" s="1">
         <v>2</v>
@@ -1898,10 +1902,10 @@
         <v>44650</v>
       </c>
       <c r="H29" s="10">
-        <v>44650</v>
+        <v>44651.87777777778</v>
       </c>
       <c r="I29" s="10">
-        <v>44650</v>
+        <v>44652.339062500003</v>
       </c>
       <c r="J29" s="1">
         <v>3</v>
@@ -1942,10 +1946,10 @@
         <v>44652</v>
       </c>
       <c r="H30" s="10">
-        <v>44652</v>
+        <v>44653.427083333336</v>
       </c>
       <c r="I30" s="10">
-        <v>44652</v>
+        <v>44653.619618055556</v>
       </c>
       <c r="J30" s="1">
         <v>0</v>
@@ -1982,10 +1986,10 @@
         <v>44651</v>
       </c>
       <c r="H31" s="10">
-        <v>44651</v>
+        <v>44653.947222222225</v>
       </c>
       <c r="I31" s="10">
-        <v>44651</v>
+        <v>44654.344108796293</v>
       </c>
       <c r="J31" s="1">
         <v>2</v>
@@ -2026,10 +2030,10 @@
         <v>44653</v>
       </c>
       <c r="H32" s="10">
-        <v>44653</v>
+        <v>44654.234027777777</v>
       </c>
       <c r="I32" s="10">
-        <v>44653</v>
+        <v>44654.534305555557</v>
       </c>
       <c r="J32" s="1">
         <v>0</v>
@@ -2066,10 +2070,10 @@
         <v>44653</v>
       </c>
       <c r="H33" s="10">
-        <v>44653</v>
+        <v>44654.652777777781</v>
       </c>
       <c r="I33" s="10">
-        <v>44653</v>
+        <v>44654.893807870372</v>
       </c>
       <c r="J33" s="1">
         <v>0</v>
@@ -2106,10 +2110,10 @@
         <v>44654</v>
       </c>
       <c r="H34" s="10">
-        <v>44654</v>
+        <v>44655.790972222225</v>
       </c>
       <c r="I34" s="10">
-        <v>44654</v>
+        <v>44655.966006944444</v>
       </c>
       <c r="J34" s="1">
         <v>0</v>
@@ -2146,10 +2150,10 @@
         <v>44656</v>
       </c>
       <c r="H35" s="10">
-        <v>44656</v>
+        <v>44656.714583333334</v>
       </c>
       <c r="I35" s="10">
-        <v>44656</v>
+        <v>44656.882916666669</v>
       </c>
       <c r="J35" s="1">
         <v>2</v>
@@ -2190,10 +2194,10 @@
         <v>44657</v>
       </c>
       <c r="H36" s="10">
-        <v>44657</v>
+        <v>44658.731944444444</v>
       </c>
       <c r="I36" s="10">
-        <v>44657</v>
+        <v>44658.822708333333</v>
       </c>
       <c r="J36" s="1">
         <v>2</v>

</xml_diff>